<commit_message>
update figure 1a/2/5 plots
</commit_message>
<xml_diff>
--- a/data/data_analysis/market_shares.xlsx
+++ b/data/data_analysis/market_shares.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62AE3D2E-5CE6-4504-B788-2F2D35451982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF78505C-FDCF-494F-B09D-8BB839F68B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supply" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="27">
   <si>
     <t>Scenario</t>
   </si>
@@ -122,6 +122,21 @@
   <si>
     <t>Literature</t>
   </si>
+  <si>
+    <t>100 Mt Baseline</t>
+  </si>
+  <si>
+    <t>500 Mt Baseline</t>
+  </si>
+  <si>
+    <t>1500 Mt Baseline</t>
+  </si>
+  <si>
+    <t>2400 Mt Baseline</t>
+  </si>
+  <si>
+    <t>4100 Mt Baseline</t>
+  </si>
 </sst>
 </file>
 
@@ -173,6 +188,20 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF001536"/>
+      <color rgb="FF486800"/>
+      <color rgb="FF93D500"/>
+      <color rgb="FF2063AC"/>
+      <color rgb="FF8AB7E9"/>
+      <color rgb="FF004639"/>
+      <color rgb="FF00AE8D"/>
+      <color rgb="FF5F1546"/>
+      <color rgb="FFC22A90"/>
+      <color rgb="FF005B70"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -245,22 +274,22 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Nothing Baseline</c:v>
+                  <c:v>100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Low Baseline</c:v>
+                  <c:v>500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>R2R Report</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>High Baseline</c:v>
+                  <c:v>1500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Excess Baseline</c:v>
+                  <c:v>2400 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4Gt Baseline</c:v>
+                  <c:v>4100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>Policy Integrity</c:v>
@@ -334,22 +363,22 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Nothing Baseline</c:v>
+                  <c:v>100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Low Baseline</c:v>
+                  <c:v>500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>R2R Report</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>High Baseline</c:v>
+                  <c:v>1500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Excess Baseline</c:v>
+                  <c:v>2400 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4Gt Baseline</c:v>
+                  <c:v>4100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>Policy Integrity</c:v>
@@ -423,22 +452,22 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Nothing Baseline</c:v>
+                  <c:v>100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Low Baseline</c:v>
+                  <c:v>500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>R2R Report</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>High Baseline</c:v>
+                  <c:v>1500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Excess Baseline</c:v>
+                  <c:v>2400 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4Gt Baseline</c:v>
+                  <c:v>4100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>Policy Integrity</c:v>
@@ -512,22 +541,22 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Nothing Baseline</c:v>
+                  <c:v>100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Low Baseline</c:v>
+                  <c:v>500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>R2R Report</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>High Baseline</c:v>
+                  <c:v>1500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Excess Baseline</c:v>
+                  <c:v>2400 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4Gt Baseline</c:v>
+                  <c:v>4100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>Policy Integrity</c:v>
@@ -622,22 +651,22 @@
               <c:strCache>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>Nothing Baseline</c:v>
+                  <c:v>100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Low Baseline</c:v>
+                  <c:v>500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>R2R Report</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>High Baseline</c:v>
+                  <c:v>1500 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Excess Baseline</c:v>
+                  <c:v>2400 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4Gt Baseline</c:v>
+                  <c:v>4100 Mt Baseline</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>Policy Integrity</c:v>
@@ -1912,9 +1941,19 @@
           <cx:tx>
             <cx:txData>
               <cx:f>_xlchart.v1.1</cx:f>
-              <cx:v>Nothing Baseline</cx:v>
+              <cx:v>100 Mt Baseline</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0047BB"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="001536"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="0"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -1924,9 +1963,19 @@
           <cx:tx>
             <cx:txData>
               <cx:f>_xlchart.v1.3</cx:f>
-              <cx:v>Low Baseline</cx:v>
+              <cx:v>500 Mt Baseline</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:srgbClr val="00B5E2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="005B70"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="1"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -1936,9 +1985,19 @@
           <cx:tx>
             <cx:txData>
               <cx:f>_xlchart.v1.5</cx:f>
-              <cx:v>High Baseline</cx:v>
+              <cx:v>1500 Mt Baseline</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C22A90"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="5F1546"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="2"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -1948,9 +2007,19 @@
           <cx:tx>
             <cx:txData>
               <cx:f>_xlchart.v1.7</cx:f>
-              <cx:v>Excess Baseline</cx:v>
+              <cx:v>2400 Mt Baseline</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:srgbClr val="00AE8D"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="004639"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="3"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -1960,9 +2029,19 @@
           <cx:tx>
             <cx:txData>
               <cx:f>_xlchart.v1.9</cx:f>
-              <cx:v>4Gt Baseline</cx:v>
+              <cx:v>4100 Mt Baseline</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:srgbClr val="8AB7E9"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2063AC"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="4"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -1975,6 +2054,16 @@
               <cx:v>Literature</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:srgbClr val="93D500"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="486800"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="5"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -1987,6 +2076,16 @@
               <cx:v>Carbon Negative Shot</cx:v>
             </cx:txData>
           </cx:tx>
+          <cx:spPr>
+            <a:solidFill>
+              <a:srgbClr val="001536"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="001536"/>
+              </a:solidFill>
+            </a:ln>
+          </cx:spPr>
           <cx:dataId val="6"/>
           <cx:layoutPr>
             <cx:statistics quartileMethod="exclusive"/>
@@ -2033,7 +2132,7 @@
         </cx:txPr>
       </cx:axis>
       <cx:axis id="1">
-        <cx:valScaling min="50"/>
+        <cx:valScaling max="750" min="50"/>
         <cx:title>
           <cx:tx>
             <cx:rich>
@@ -3944,7 +4043,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="4524374" y="2262186"/>
+              <a:off x="5133974" y="2262186"/>
               <a:ext cx="9667875" cy="4329113"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -4319,7 +4418,7 @@
         <v>8100</v>
       </c>
       <c r="K3" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="L3">
         <v>100</v>
@@ -4363,7 +4462,7 @@
         <v>33.333333333333336</v>
       </c>
       <c r="K4" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="L4">
         <v>500</v>
@@ -4451,7 +4550,7 @@
         <v>18.518518518518519</v>
       </c>
       <c r="K6" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="L6">
         <v>1500</v>
@@ -4495,7 +4594,7 @@
         <v>19.753086419753089</v>
       </c>
       <c r="K7" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="L7">
         <v>2400</v>
@@ -4515,7 +4614,7 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="K8" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="L8">
         <v>4100</v>
@@ -4785,19 +4884,19 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
         <v>21</v>

</xml_diff>